<commit_message>
Lekce 1.1: screenshoty před a po a kontrola střediska IT
</commit_message>
<xml_diff>
--- a/01_excel/lekce_1_1_naklady.xlsx
+++ b/01_excel/lekce_1_1_naklady.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucia\Documents\data_analytika\01_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E44F6127-F708-4F3F-A620-97EB3B36696B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B8904BB-B84D-4BED-8DC1-52FED8524492}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -270,17 +270,17 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -683,44 +683,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="15" t="s">
+      <c r="A4" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="15"/>
-      <c r="E4" s="15"/>
-      <c r="F4" s="15" t="s">
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="16" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="15"/>
-      <c r="B5" s="15"/>
+      <c r="A5" s="16"/>
+      <c r="B5" s="16"/>
       <c r="C5" s="3" t="s">
         <v>16</v>
       </c>
@@ -730,11 +730,11 @@
       <c r="E5" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="F5" s="15"/>
+      <c r="F5" s="16"/>
       <c r="H5" s="11"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="16" t="s">
+      <c r="A6" s="14" t="s">
         <v>19</v>
       </c>
       <c r="B6" s="4" t="s">
@@ -755,7 +755,7 @@
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="17"/>
+      <c r="A7" s="15"/>
       <c r="B7" s="4" t="s">
         <v>21</v>
       </c>
@@ -774,7 +774,7 @@
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="17"/>
+      <c r="A8" s="15"/>
       <c r="B8" s="4" t="s">
         <v>22</v>
       </c>
@@ -823,7 +823,7 @@
       <c r="F10" s="4"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11" s="16" t="s">
+      <c r="A11" s="14" t="s">
         <v>24</v>
       </c>
       <c r="B11" s="4" t="s">
@@ -844,7 +844,7 @@
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" s="17"/>
+      <c r="A12" s="15"/>
       <c r="B12" s="4" t="s">
         <v>21</v>
       </c>
@@ -863,7 +863,7 @@
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A13" s="17"/>
+      <c r="A13" s="15"/>
       <c r="B13" s="4" t="s">
         <v>22</v>
       </c>
@@ -912,7 +912,7 @@
       <c r="F15" s="4"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A16" s="16" t="s">
+      <c r="A16" s="14" t="s">
         <v>27</v>
       </c>
       <c r="B16" s="4" t="s">
@@ -933,7 +933,7 @@
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="17"/>
+      <c r="A17" s="15"/>
       <c r="B17" s="4" t="s">
         <v>21</v>
       </c>
@@ -952,7 +952,7 @@
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="17"/>
+      <c r="A18" s="15"/>
       <c r="B18" s="4" t="s">
         <v>22</v>
       </c>
@@ -1016,10 +1016,7 @@
       <c r="A23" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="F23" s="19">
-        <f>SUM(F9,F14,F19)+34000</f>
-        <v>3813450</v>
-      </c>
+      <c r="F23" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -1078,7 +1075,7 @@
       <c r="D2" t="s">
         <v>37</v>
       </c>
-      <c r="E2" s="19">
+      <c r="E2" s="13">
         <v>18400</v>
       </c>
     </row>
@@ -1095,10 +1092,10 @@
       <c r="D3" t="s">
         <v>38</v>
       </c>
-      <c r="E3" s="19">
+      <c r="E3" s="13">
         <v>86500</v>
       </c>
-      <c r="G3" s="19"/>
+      <c r="G3" s="13"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="12">
@@ -1113,7 +1110,7 @@
       <c r="D4" t="s">
         <v>39</v>
       </c>
-      <c r="E4" s="19">
+      <c r="E4" s="13">
         <v>412000</v>
       </c>
     </row>
@@ -1130,7 +1127,7 @@
       <c r="D5" t="s">
         <v>37</v>
       </c>
-      <c r="E5" s="19">
+      <c r="E5" s="13">
         <v>6200</v>
       </c>
     </row>
@@ -1147,7 +1144,7 @@
       <c r="D6" t="s">
         <v>38</v>
       </c>
-      <c r="E6" s="19">
+      <c r="E6" s="13">
         <v>34000</v>
       </c>
     </row>
@@ -1164,7 +1161,7 @@
       <c r="D7" t="s">
         <v>39</v>
       </c>
-      <c r="E7" s="19">
+      <c r="E7" s="13">
         <v>268000</v>
       </c>
     </row>
@@ -1181,7 +1178,7 @@
       <c r="D8" t="s">
         <v>37</v>
       </c>
-      <c r="E8" s="19">
+      <c r="E8" s="13">
         <v>12700</v>
       </c>
     </row>
@@ -1198,7 +1195,7 @@
       <c r="D9" t="s">
         <v>38</v>
       </c>
-      <c r="E9" s="19">
+      <c r="E9" s="13">
         <v>58300</v>
       </c>
     </row>
@@ -1215,7 +1212,7 @@
       <c r="D10" t="s">
         <v>39</v>
       </c>
-      <c r="E10" s="19">
+      <c r="E10" s="13">
         <v>356000</v>
       </c>
     </row>
@@ -1232,7 +1229,7 @@
       <c r="D11" t="s">
         <v>37</v>
       </c>
-      <c r="E11" s="19">
+      <c r="E11" s="13">
         <v>22150</v>
       </c>
     </row>
@@ -1249,7 +1246,7 @@
       <c r="D12" t="s">
         <v>38</v>
       </c>
-      <c r="E12" s="19">
+      <c r="E12" s="13">
         <v>91200</v>
       </c>
     </row>
@@ -1266,7 +1263,7 @@
       <c r="D13" t="s">
         <v>39</v>
       </c>
-      <c r="E13" s="19">
+      <c r="E13" s="13">
         <v>412000</v>
       </c>
     </row>
@@ -1283,7 +1280,7 @@
       <c r="D14" t="s">
         <v>37</v>
       </c>
-      <c r="E14" s="19">
+      <c r="E14" s="13">
         <v>4850</v>
       </c>
     </row>
@@ -1300,7 +1297,7 @@
       <c r="D15" t="s">
         <v>38</v>
       </c>
-      <c r="E15" s="19">
+      <c r="E15" s="13">
         <v>29500</v>
       </c>
     </row>
@@ -1317,7 +1314,7 @@
       <c r="D16" t="s">
         <v>39</v>
       </c>
-      <c r="E16" s="19">
+      <c r="E16" s="13">
         <v>268000</v>
       </c>
     </row>
@@ -1334,7 +1331,7 @@
       <c r="D17" t="s">
         <v>37</v>
       </c>
-      <c r="E17" s="19">
+      <c r="E17" s="13">
         <v>14300</v>
       </c>
     </row>
@@ -1351,7 +1348,7 @@
       <c r="D18" t="s">
         <v>38</v>
       </c>
-      <c r="E18" s="19">
+      <c r="E18" s="13">
         <v>62900</v>
       </c>
     </row>
@@ -1368,7 +1365,7 @@
       <c r="D19" t="s">
         <v>39</v>
       </c>
-      <c r="E19" s="19">
+      <c r="E19" s="13">
         <v>361500</v>
       </c>
     </row>
@@ -1385,7 +1382,7 @@
       <c r="D20" t="s">
         <v>37</v>
       </c>
-      <c r="E20" s="19">
+      <c r="E20" s="13">
         <v>15900</v>
       </c>
     </row>
@@ -1402,7 +1399,7 @@
       <c r="D21" t="s">
         <v>38</v>
       </c>
-      <c r="E21" s="19">
+      <c r="E21" s="13">
         <v>88700</v>
       </c>
     </row>
@@ -1419,7 +1416,7 @@
       <c r="D22" t="s">
         <v>39</v>
       </c>
-      <c r="E22" s="19">
+      <c r="E22" s="13">
         <v>425600</v>
       </c>
     </row>
@@ -1436,7 +1433,7 @@
       <c r="D23" t="s">
         <v>37</v>
       </c>
-      <c r="E23" s="19">
+      <c r="E23" s="13">
         <v>7300</v>
       </c>
     </row>
@@ -1453,7 +1450,7 @@
       <c r="D24" t="s">
         <v>38</v>
       </c>
-      <c r="E24" s="19">
+      <c r="E24" s="13">
         <v>41200</v>
       </c>
     </row>
@@ -1470,7 +1467,7 @@
       <c r="D25" t="s">
         <v>39</v>
       </c>
-      <c r="E25" s="19">
+      <c r="E25" s="13">
         <v>271400</v>
       </c>
     </row>
@@ -1487,7 +1484,7 @@
       <c r="D26" t="s">
         <v>37</v>
       </c>
-      <c r="E26" s="19">
+      <c r="E26" s="13">
         <v>11900</v>
       </c>
     </row>
@@ -1504,7 +1501,7 @@
       <c r="D27" t="s">
         <v>38</v>
       </c>
-      <c r="E27" s="19">
+      <c r="E27" s="13">
         <v>71450</v>
       </c>
     </row>
@@ -1521,7 +1518,7 @@
       <c r="D28" t="s">
         <v>39</v>
       </c>
-      <c r="E28" s="19">
+      <c r="E28" s="13">
         <v>361500</v>
       </c>
     </row>
@@ -1532,7 +1529,7 @@
       <c r="B29" s="10"/>
       <c r="C29" s="10"/>
       <c r="D29" s="10"/>
-      <c r="E29" s="19">
+      <c r="E29" s="13">
         <f>SUBTOTAL(109,tbl_Naklady[Castka])</f>
         <v>1572450</v>
       </c>

</xml_diff>